<commit_message>
📊 BIST Screener | 04.05.2026 16:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-04.xlsx
+++ b/data/bist_screener_2026-05-04.xlsx
@@ -25789,79 +25789,67 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>145</v>
+        <v>240.3</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0335</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>2230000</v>
+        <v>7350</v>
       </c>
       <c r="E583" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.2578</v>
       </c>
       <c r="F583" s="7" t="n">
-        <v>49.45</v>
+        <v>40.8</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J583" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I583" s="6" t="inlineStr"/>
+      <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>63.5</v>
+        <v>162.4</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0283</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>690340</v>
-      </c>
-      <c r="E584" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>6590000</v>
+      </c>
+      <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>53.19</v>
+        <v>55.37</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="2" t="inlineStr"/>
-      <c r="J584" s="4" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25869,40 +25857,34 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>2.69</v>
+        <v>18.58</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0037</v>
+        <v>-0.0226</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>84710000</v>
-      </c>
-      <c r="E585" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>54870000</v>
+      </c>
+      <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>42.8</v>
+        <v>27.79</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J585" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I585" s="6" t="inlineStr"/>
+      <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25910,21 +25892,23 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>33.14</v>
+        <v>30.2</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0024</v>
-      </c>
-      <c r="D586" s="3" t="n">
-        <v>4190000</v>
-      </c>
-      <c r="E586" s="2" t="inlineStr"/>
+        <v>0.0604</v>
+      </c>
+      <c r="D586" s="5" t="n">
+        <v>18980000</v>
+      </c>
+      <c r="E586" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F586" s="3" t="n">
-        <v>48.62</v>
+        <v>56.55</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25932,12 +25916,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25945,21 +25929,23 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>14.1</v>
+        <v>6.24</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0086</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>31090000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>61950000</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>55.39</v>
+        <v>88.19</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25967,12 +25953,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25980,34 +25966,40 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>17.25</v>
+        <v>145</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0141</v>
+        <v>0.0335</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>67270000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>2230000</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>53.71</v>
+        <v>49.45</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -26015,23 +26007,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>6.24</v>
+        <v>86</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.09859999999999999</v>
+        <v>-0.06619999999999999</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>61950000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>221580</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>88.19</v>
+        <v>10.99</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26042,31 +26032,27 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
-        </is>
-      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>39.08</v>
+        <v>17.25</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.0141</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>10030000</v>
+        <v>67270000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>49.97</v>
+        <v>53.71</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26074,12 +26060,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26087,34 +26073,40 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>20.94</v>
+        <v>2.69</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0242</v>
+        <v>0.0037</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>88110000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>84710000</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>66.18000000000001</v>
+        <v>42.8</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26122,21 +26114,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>18.58</v>
+        <v>29.86</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0226</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>54870000</v>
+        <v>19130000</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>27.79</v>
+        <v>70.78</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26144,12 +26136,12 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26157,36 +26149,28 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>40.7</v>
+        <v>79.48999999999999</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.003</v>
+        <v>-0.0129</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>7140000</v>
+        <v>10820000</v>
       </c>
       <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>54.7</v>
+        <v>39.95</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
       <c r="J593" s="6" t="inlineStr"/>
-      <c r="K593" s="6" t="inlineStr">
-        <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+      <c r="K593" s="6" t="inlineStr"/>
+      <c r="L593" s="6" t="inlineStr"/>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
@@ -26235,139 +26219,143 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>190</v>
+        <v>6.47</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0026</v>
+        <v>-0.0757</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>18260000</v>
-      </c>
-      <c r="E595" s="6" t="inlineStr"/>
+        <v>730100</v>
+      </c>
+      <c r="E595" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F595" s="7" t="n">
-        <v>45.2</v>
+        <v>33.73</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="6" t="inlineStr"/>
+      <c r="I595" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J595" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr"/>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>6.47</v>
+        <v>33.14</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.0757</v>
-      </c>
-      <c r="D596" s="5" t="n">
-        <v>730100</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>0.0024</v>
+      </c>
+      <c r="D596" s="3" t="n">
+        <v>4190000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>33.73</v>
+        <v>48.62</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J596" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I596" s="2" t="inlineStr"/>
+      <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>79.48999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0129</v>
+        <v>0.0968</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>10820000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>44050</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>39.95</v>
+        <v>53.3</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
-      <c r="K597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-4.155</v>
+      </c>
+      <c r="K597" s="6" t="inlineStr">
+        <is>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
       <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>18.13</v>
+        <v>40.7</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0106</v>
+        <v>0.003</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.9869</v>
-      </c>
+        <v>7140000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>59.1</v>
+        <v>54.7</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="4" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J598" s="4" t="n">
-        <v>0.3246</v>
-      </c>
+      <c r="I598" s="2" t="inlineStr"/>
+      <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26375,122 +26363,138 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>86.09999999999999</v>
+        <v>20.94</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0968</v>
+        <v>-0.0242</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>44050</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>88110000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>53.3</v>
+        <v>66.18000000000001</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J599" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I599" s="6" t="inlineStr"/>
+      <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr"/>
+          <t>Ticari hizmetler</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+        </is>
+      </c>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>240.3</v>
+        <v>18.13</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.0106</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>7350</v>
+        <v>1180000</v>
       </c>
       <c r="E600" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.9869</v>
       </c>
       <c r="F600" s="3" t="n">
-        <v>40.8</v>
+        <v>59.1</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
+      <c r="I600" s="4" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J600" s="4" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L600" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L600" s="2" t="inlineStr">
+        <is>
+          <t>BIST MENKUL KIYM YO</t>
+        </is>
+      </c>
       <c r="M600" s="2" t="inlineStr"/>
     </row>
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>6.17</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0016</v>
+        <v>0.09970000000000001</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>7970000</v>
-      </c>
-      <c r="E601" s="6" t="inlineStr"/>
+        <v>104590000</v>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F601" s="7" t="n">
-        <v>63.63</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
         </is>
       </c>
-      <c r="L601" s="6" t="inlineStr"/>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>86</v>
+        <v>14.1</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.06619999999999999</v>
+        <v>0.0086</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>221580</v>
+        <v>31090000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>10.99</v>
+        <v>55.39</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26498,32 +26502,34 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr"/>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>30.2</v>
+        <v>2.88</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0604</v>
+        <v>-0.0204</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>18980000</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>243030000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>56.55</v>
+        <v>53.45</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26531,12 +26537,12 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26544,21 +26550,21 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>2.88</v>
+        <v>190</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0204</v>
+        <v>0.0026</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>243030000</v>
+        <v>18260000</v>
       </c>
       <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>53.45</v>
+        <v>45.2</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
@@ -26566,12 +26572,12 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26579,75 +26585,69 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>8.380000000000001</v>
+        <v>6.17</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.09970000000000001</v>
+        <v>0.0016</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>104590000</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>7970000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>73.98999999999999</v>
+        <v>63.63</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
       <c r="K605" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
         </is>
       </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>162.4</v>
+        <v>63.5</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>-0.0283</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>6590000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>690340</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>55.37</v>
+        <v>53.19</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="2" t="inlineStr"/>
+      <c r="J606" s="4" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26655,21 +26655,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>29.86</v>
+        <v>39.08</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.009300000000000001</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>19130000</v>
+        <v>10030000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>70.78</v>
+        <v>49.97</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26677,12 +26677,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26709,7 +26709,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>04.05.2026 15:30</t>
+          <t>04.05.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 04.05.2026 17:10 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-04.xlsx
+++ b/data/bist_screener_2026-05-04.xlsx
@@ -25789,23 +25789,21 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>240.3</v>
+        <v>17.25</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>-0.006999999999999999</v>
+        <v>0.0141</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>7350</v>
-      </c>
-      <c r="E583" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>67270000</v>
+      </c>
+      <c r="E583" s="6" t="inlineStr"/>
       <c r="F583" s="7" t="n">
-        <v>40.8</v>
+        <v>53.71</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
@@ -25813,30 +25811,34 @@
       <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>162.4</v>
+        <v>29.86</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>0.09939999999999999</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>6590000</v>
+        <v>19130000</v>
       </c>
       <c r="E584" s="2" t="inlineStr"/>
       <c r="F584" s="3" t="n">
-        <v>55.37</v>
+        <v>70.78</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25844,12 +25846,12 @@
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25857,21 +25859,21 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>18.58</v>
+        <v>6.17</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.0226</v>
+        <v>0.0016</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>54870000</v>
+        <v>7970000</v>
       </c>
       <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>27.79</v>
+        <v>63.63</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
@@ -25882,33 +25884,27 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L585" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="L585" s="6" t="inlineStr"/>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>30.2</v>
+        <v>20.94</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0604</v>
+        <v>-0.0242</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>18980000</v>
-      </c>
-      <c r="E586" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>88110000</v>
+      </c>
+      <c r="E586" s="2" t="inlineStr"/>
       <c r="F586" s="3" t="n">
-        <v>56.55</v>
+        <v>66.18000000000001</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
@@ -25916,12 +25912,12 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25929,36 +25925,40 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>6.24</v>
+        <v>2.69</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.0037</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>61950000</v>
+        <v>84710000</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.7119</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>88.19</v>
+        <v>42.8</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="I587" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J587" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25966,40 +25966,34 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>145</v>
+        <v>14.1</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0335</v>
+        <v>0.0086</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>2230000</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>31090000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>49.45</v>
+        <v>55.39</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J588" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -26007,52 +26001,66 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>86</v>
+        <v>17.11</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.06619999999999999</v>
+        <v>0.0035</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>221580</v>
-      </c>
-      <c r="E589" s="6" t="inlineStr"/>
+        <v>11260000</v>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F589" s="7" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G589" s="6" t="inlineStr"/>
+        <v>47.32</v>
+      </c>
+      <c r="G589" s="7" t="n">
+        <v>161.72</v>
+      </c>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="6" t="inlineStr"/>
-      <c r="J589" s="6" t="inlineStr"/>
+      <c r="I589" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J589" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+        </is>
+      </c>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>17.25</v>
+        <v>6.24</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0141</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>67270000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>61950000</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>53.71</v>
+        <v>88.19</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26065,7 +26073,7 @@
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26073,40 +26081,38 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>2.69</v>
+        <v>63.5</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0037</v>
+        <v>-0.0283</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>84710000</v>
+        <v>690340</v>
       </c>
       <c r="E591" s="8" t="n">
-        <v>0.7119</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F591" s="7" t="n">
-        <v>42.8</v>
+        <v>53.19</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
       <c r="J591" s="8" t="n">
-        <v>-0.8093</v>
+        <v>0.4139</v>
       </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26114,21 +26120,21 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>29.86</v>
+        <v>86</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.09939999999999999</v>
+        <v>-0.06619999999999999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>19130000</v>
+        <v>221580</v>
       </c>
       <c r="E592" s="2" t="inlineStr"/>
       <c r="F592" s="3" t="n">
-        <v>70.78</v>
+        <v>10.99</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
@@ -26136,82 +26142,84 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>79.48999999999999</v>
+        <v>18.13</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0129</v>
+        <v>0.0106</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>10820000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>1180000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>39.95</v>
+        <v>59.1</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
-      <c r="K593" s="6" t="inlineStr"/>
-      <c r="L593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>0.3246</v>
+      </c>
+      <c r="K593" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST MENKUL KIYM YO</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>17.11</v>
+        <v>162.4</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0035</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>11260000</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>6590000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>47.32</v>
-      </c>
-      <c r="G594" s="3" t="n">
-        <v>161.72</v>
-      </c>
+        <v>55.37</v>
+      </c>
+      <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26219,58 +26227,56 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>6.47</v>
+        <v>33.14</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0757</v>
-      </c>
-      <c r="D595" s="9" t="n">
-        <v>730100</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>0.0024</v>
+      </c>
+      <c r="D595" s="7" t="n">
+        <v>4190000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>33.73</v>
+        <v>48.62</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J595" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>33.14</v>
+        <v>2.88</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0024</v>
-      </c>
-      <c r="D596" s="3" t="n">
-        <v>4190000</v>
+        <v>-0.0204</v>
+      </c>
+      <c r="D596" s="5" t="n">
+        <v>243030000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>48.62</v>
+        <v>53.45</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26278,12 +26284,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26291,139 +26297,135 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>86.09999999999999</v>
+        <v>40.7</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0968</v>
+        <v>0.003</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>44050</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.58</v>
-      </c>
+        <v>7140000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>53.3</v>
+        <v>54.7</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>40.7</v>
+        <v>6.47</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.003</v>
+        <v>-0.0757</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>7140000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>730100</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>54.7</v>
+        <v>33.73</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J598" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr"/>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>20.94</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>-0.0242</v>
+        <v>0.0968</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>88110000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>44050</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>66.18000000000001</v>
+        <v>53.3</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="6" t="inlineStr"/>
+      <c r="I599" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J599" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>18.13</v>
+        <v>18.58</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0106</v>
+        <v>-0.0226</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>1180000</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.9869</v>
-      </c>
+        <v>54870000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>59.1</v>
+        <v>27.79</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
-      <c r="I600" s="4" t="n">
-        <v>-0.2446</v>
-      </c>
-      <c r="J600" s="4" t="n">
-        <v>0.3246</v>
-      </c>
+      <c r="I600" s="2" t="inlineStr"/>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26431,7 +26433,7 @@
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26439,40 +26441,36 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>8.380000000000001</v>
+        <v>30.2</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.09970000000000001</v>
+        <v>0.0604</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>104590000</v>
+        <v>18980000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.2667</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>73.98999999999999</v>
+        <v>56.55</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26480,21 +26478,21 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>14.1</v>
+        <v>190</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0086</v>
+        <v>0.0026</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>31090000</v>
+        <v>18260000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>55.39</v>
+        <v>45.2</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26502,12 +26500,12 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26515,34 +26513,40 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>2.88</v>
+        <v>145</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>-0.0204</v>
+        <v>0.0335</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>243030000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>2230000</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>53.45</v>
+        <v>49.45</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="6" t="inlineStr"/>
-      <c r="J603" s="6" t="inlineStr"/>
+      <c r="I603" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J603" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26550,34 +26554,40 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>190</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0026</v>
+        <v>0.09970000000000001</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>18260000</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>104590000</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.1672</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>45.2</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J604" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26585,71 +26595,61 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>6.17</v>
+        <v>79.48999999999999</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0016</v>
+        <v>-0.0129</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>7970000</v>
+        <v>10820000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>63.63</v>
+        <v>39.95</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
       <c r="J605" s="6" t="inlineStr"/>
-      <c r="K605" s="6" t="inlineStr">
-        <is>
-          <t>Finans</t>
-        </is>
-      </c>
+      <c r="K605" s="6" t="inlineStr"/>
       <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>63.5</v>
+        <v>240.3</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0283</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>690340</v>
+        <v>7350</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.2578</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>53.19</v>
+        <v>40.8</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="2" t="inlineStr"/>
-      <c r="J606" s="4" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
@@ -26709,7 +26709,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>04.05.2026 16:30</t>
+          <t>04.05.2026 17:10</t>
         </is>
       </c>
     </row>

</xml_diff>